<commit_message>
docs: reconcile README, diagrams, data dictionary and report with the code
- Redraw docs/architecture.png (five DAG tasks, validation gate, separate
  rejected-record and validation-issue files, loading stage, real Part 2 flow,
  Docker tested with a synthetic bundle only) and docs/Schema_Diagram.png
  (exact columns, types, keys, NOT NULL and all five foreign keys).
- Validation Rules sheet now lists the nine implemented checks, the cleaning
  rules and the exit-code gate; evidence sheet is dated.
- README and report: nine checks, validation_issues.csv vs rejected_records.csv,
  IDS mapping and diagnosis unpivot in loading, Airflow deployment and evidence
  dates, read-only row-count check, 258-test run and the known flaky test.
- Report PDF re-printed from the HTML (9 pages).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data_dictionary.xlsx
+++ b/docs/data_dictionary.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Rules" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Evidence" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Data Dictionary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Validation Rules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Current Evidence" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Dictionary'!$A$1:$D$37</definedName>
@@ -1268,12 +1268,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1296,170 +1296,255 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Primary keys</t>
+          <t>Cleaning (clean.py)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Encounter ID in admissions is unique and non-null</t>
+          <t>Rows missing encounter_id or patient_nbr are removed</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>No duplicate/null encounter IDs</t>
+          <t>Removed rows written to logs/validation/rejected_records.csv (header only if none)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Primary keys</t>
+          <t>Cleaning (clean.py)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Patient SK in patient_summary is unique and non-null</t>
+          <t>Duplicate encounter_id rows are removed (first kept)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>No duplicate/null patient keys</t>
+          <t>Removed rows written to logs/validation/rejected_records.csv</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Surrogate keys</t>
+          <t>Cleaning (clean.py)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>COUNT(*) equals COUNT(DISTINCT patient_sk) in patient_summary</t>
+          <t>'?' missing-value codes replaced by true missing values</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Duplicate patient keys = 0</t>
+          <t>Consistent missing-value representation</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Foreign keys</t>
+          <t>Validation check 1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Curated foreign-key relationships must reference existing parent records</t>
+          <t>encounter_id and patient_sk present in the cleaned file</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>All references valid</t>
+          <t>No missing identifiers</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Readmission flag</t>
+          <t>Validation check 2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>readmitted_within_30_days represents the 30-day readmission indicator</t>
+          <t>encounter_id is unique in the cleaned file</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Valid readmission status values</t>
+          <t>Duplicate encounter IDs = 0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Length of stay</t>
+          <t>Validation check 3</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>length_of_stay_days should be non-negative</t>
+          <t>No '?' code remains in the cleaned file</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>No negative LOS values</t>
+          <t>Special missing-value codes = 0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Validation check 4</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Diagnosis, medication and encounter counts should be non-negative</t>
+          <t>readmitted is one of NO, &lt;30, &gt;30</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>No negative count values</t>
+          <t>Invalid readmission categories = 0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Duplicates</t>
+          <t>Validation check 5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Duplicate encounters are removed during cleaning</t>
+          <t>time_in_hospital is between 1 and 14 days</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>One curated row per encounter</t>
+          <t>Out-of-range length of stay = 0</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Missing values</t>
+          <t>Validation check 6</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Special missing-value codes are standardized during cleaning</t>
+          <t>prior_admission is 0 or 1 (analytical file)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Consistent missing-value representation</t>
+          <t>Invalid prior_admission values = 0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Invalid records</t>
+          <t>Validation check 7</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Invalid encounters are rejected and recorded</t>
+          <t>diagnosis_count is between 0 and 3 (analytical file)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Rejected/error records logged</t>
+          <t>Out-of-range diagnosis counts = 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Validation check 8</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>medication_count is between 0 and 23 (analytical file)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Out-of-range medication counts = 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Validation check 9</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Cleaned and analytical files have the same row count</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Row counts equal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Validation outcome</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Any failed check: validate.py exits with code 1; Airflow marks validation failed and does not run postgresql_loading</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>All 9 checks pass: exit code 0 and loading runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Validation outputs</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>One row per failed check (check, message, count) in logs/validation/validation_issues.csv; status in validation_log.txt</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Header-only issues file when all checks pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Database (schema.sql)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Primary keys, NOT NULL keys and 5 foreign keys enforced by PostgreSQL during loading</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Load fails and rolls back on a violation</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1590,6 +1675,30 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Evidence source</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Read-only query of database hospital_readmission</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Evidence date</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>15 Oct 2026 (re-confirmed; same values as the 6 Sep 2026 load)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>